<commit_message>
Excel book: revised edition (beginner to intermediate), unified chapter structure, quizzes and solutions, zoomed figures, formula tests, revision report and sales page
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0119EEHr9PMFFRyRJjMJGbmM
</commit_message>
<xml_diff>
--- a/docs/excel-book/projets/Exercices-par-chapitre.xlsx
+++ b/docs/excel-book/projets/Exercices-par-chapitre.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="75">
   <si>
     <t xml:space="preserve">Chapitre 5 · Formules et références</t>
   </si>
@@ -68,9 +68,6 @@
     <t xml:space="preserve">Trousse</t>
   </si>
   <si>
-    <t xml:space="preserve">Solution : D6 =B6*C6 · E6 =D6*$F$3 · F6 =D6+E6, puis recopiez vers le bas.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Chapitres 6 et 7 · Fonctions</t>
   </si>
   <si>
@@ -177,9 +174,6 @@
   </si>
   <si>
     <t xml:space="preserve">Prix :</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Solution : =RECHERCHEV(B13;A5:D10;2;FAUX) puis colonne 3 pour le prix.</t>
   </si>
   <si>
     <t xml:space="preserve">Chapitre 9 · Texte et dates</t>
@@ -431,7 +425,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -476,11 +470,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -867,9 +869,7 @@
       <c r="F10" s="8"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
-        <v>14</v>
-      </c>
+      <c r="A12" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -902,7 +902,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -911,7 +911,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -920,27 +920,27 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>20</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="10" t="s">
         <v>22</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>23</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>120000</v>
@@ -952,10 +952,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>98000</v>
@@ -967,10 +967,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>25</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>26</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>76000</v>
@@ -982,10 +982,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>143000</v>
@@ -997,10 +997,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>54000</v>
@@ -1012,10 +1012,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>110000</v>
@@ -1027,39 +1027,39 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D12" s="8"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D13" s="8"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D14" s="8"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="D15" s="8"/>
+        <v>32</v>
+      </c>
+      <c r="D15" s="13"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D16" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="D17" s="8"/>
+        <v>34</v>
+      </c>
+      <c r="D17" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1090,7 +1090,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1098,7 +1098,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1106,7 +1106,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>3</v>
@@ -1115,12 +1115,12 @@
         <v>4</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>9</v>
@@ -1134,7 +1134,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>10</v>
@@ -1148,7 +1148,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>11</v>
@@ -1162,10 +1162,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="10" t="s">
         <v>43</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>44</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>750</v>
@@ -1176,7 +1176,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>12</v>
@@ -1190,10 +1190,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>46</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>47</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>1200</v>
@@ -1204,28 +1204,26 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>49</v>
-      </c>
-      <c r="B14" s="11"/>
+        <v>48</v>
+      </c>
+      <c r="B14" s="14"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B15" s="8"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="9" t="s">
-        <v>51</v>
-      </c>
+      <c r="A17" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1260,7 +1258,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1270,7 +1268,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1280,71 +1278,71 @@
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C4" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="D4" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>58</v>
-      </c>
       <c r="F4" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="13" t="n">
+        <v>57</v>
+      </c>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="15" t="n">
         <v>35868</v>
       </c>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="13" t="n">
+        <v>58</v>
+      </c>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="15" t="n">
         <v>37197</v>
       </c>
-      <c r="E6" s="11"/>
-      <c r="F6" s="11"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="13" t="n">
+        <v>59</v>
+      </c>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="15" t="n">
         <v>34903</v>
       </c>
-      <c r="E7" s="11"/>
-      <c r="F7" s="11"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>62</v>
-      </c>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="13" t="n">
+        <v>60</v>
+      </c>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="15" t="n">
         <v>37651</v>
       </c>
-      <c r="E8" s="11"/>
-      <c r="F8" s="11"/>
+      <c r="E8" s="14"/>
+      <c r="F8" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1376,7 +1374,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1385,7 +1383,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1394,10 +1392,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>3</v>
@@ -1406,18 +1404,18 @@
         <v>5</v>
       </c>
       <c r="E4" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="15" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>67</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="n">
-        <v>46137</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>69</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>13</v>
@@ -1427,14 +1425,14 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="n">
+      <c r="A6" s="15" t="n">
         <v>46123</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>10</v>
@@ -1444,14 +1442,14 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="n">
+      <c r="A7" s="15" t="n">
         <v>46199</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D7" s="7" t="n">
         <v>44</v>
@@ -1461,14 +1459,14 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13" t="n">
+      <c r="A8" s="15" t="n">
         <v>46118</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D8" s="7" t="n">
         <v>7</v>
@@ -1478,14 +1476,14 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="n">
+      <c r="A9" s="15" t="n">
         <v>46148</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D9" s="7" t="n">
         <v>12</v>
@@ -1495,14 +1493,14 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="n">
+      <c r="A10" s="15" t="n">
         <v>46077</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D10" s="7" t="n">
         <v>40</v>
@@ -1512,14 +1510,14 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="n">
+      <c r="A11" s="15" t="n">
         <v>46200</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D11" s="7" t="n">
         <v>29</v>
@@ -1529,14 +1527,14 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="n">
+      <c r="A12" s="15" t="n">
         <v>46170</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D12" s="7" t="n">
         <v>24</v>
@@ -1546,14 +1544,14 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="n">
+      <c r="A13" s="15" t="n">
         <v>46125</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D13" s="7" t="n">
         <v>37</v>
@@ -1563,14 +1561,14 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13" t="n">
+      <c r="A14" s="15" t="n">
         <v>46054</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D14" s="7" t="n">
         <v>34</v>
@@ -1580,14 +1578,14 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="n">
+      <c r="A15" s="15" t="n">
         <v>46137</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>58</v>
@@ -1597,14 +1595,14 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="n">
+      <c r="A16" s="15" t="n">
         <v>46125</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D16" s="7" t="n">
         <v>13</v>
@@ -1614,14 +1612,14 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="n">
+      <c r="A17" s="15" t="n">
         <v>46124</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D17" s="7" t="n">
         <v>37</v>
@@ -1631,14 +1629,14 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="n">
+      <c r="A18" s="15" t="n">
         <v>46043</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D18" s="7" t="n">
         <v>51</v>
@@ -1648,14 +1646,14 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="n">
+      <c r="A19" s="15" t="n">
         <v>46190</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D19" s="7" t="n">
         <v>53</v>
@@ -1665,14 +1663,14 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="n">
+      <c r="A20" s="15" t="n">
         <v>46199</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D20" s="7" t="n">
         <v>59</v>
@@ -1682,14 +1680,14 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13" t="n">
+      <c r="A21" s="15" t="n">
         <v>46166</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D21" s="7" t="n">
         <v>13</v>
@@ -1699,14 +1697,14 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13" t="n">
+      <c r="A22" s="15" t="n">
         <v>46107</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D22" s="7" t="n">
         <v>9</v>
@@ -1716,14 +1714,14 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="13" t="n">
+      <c r="A23" s="15" t="n">
         <v>46167</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D23" s="7" t="n">
         <v>25</v>
@@ -1733,14 +1731,14 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="13" t="n">
+      <c r="A24" s="15" t="n">
         <v>46117</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D24" s="7" t="n">
         <v>18</v>
@@ -1750,14 +1748,14 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="n">
+      <c r="A25" s="15" t="n">
         <v>46159</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D25" s="7" t="n">
         <v>28</v>
@@ -1767,14 +1765,14 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="13" t="n">
+      <c r="A26" s="15" t="n">
         <v>46059</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D26" s="7" t="n">
         <v>45</v>
@@ -1784,14 +1782,14 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="13" t="n">
+      <c r="A27" s="15" t="n">
         <v>46184</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D27" s="7" t="n">
         <v>55</v>
@@ -1801,14 +1799,14 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13" t="n">
+      <c r="A28" s="15" t="n">
         <v>46047</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D28" s="7" t="n">
         <v>45</v>
@@ -1818,14 +1816,14 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="13" t="n">
+      <c r="A29" s="15" t="n">
         <v>46130</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D29" s="7" t="n">
         <v>21</v>
@@ -1835,14 +1833,14 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="13" t="n">
+      <c r="A30" s="15" t="n">
         <v>46199</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D30" s="7" t="n">
         <v>29</v>
@@ -1852,14 +1850,14 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="13" t="n">
+      <c r="A31" s="15" t="n">
         <v>46147</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D31" s="7" t="n">
         <v>53</v>
@@ -1869,14 +1867,14 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="13" t="n">
+      <c r="A32" s="15" t="n">
         <v>46120</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D32" s="7" t="n">
         <v>23</v>
@@ -1886,14 +1884,14 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="13" t="n">
+      <c r="A33" s="15" t="n">
         <v>46102</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D33" s="7" t="n">
         <v>51</v>
@@ -1903,14 +1901,14 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="13" t="n">
+      <c r="A34" s="15" t="n">
         <v>46175</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D34" s="7" t="n">
         <v>23</v>
@@ -1920,14 +1918,14 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="13" t="n">
+      <c r="A35" s="15" t="n">
         <v>46129</v>
       </c>
       <c r="B35" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D35" s="7" t="n">
         <v>13</v>
@@ -1937,14 +1935,14 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="13" t="n">
+      <c r="A36" s="15" t="n">
         <v>46073</v>
       </c>
       <c r="B36" s="10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D36" s="7" t="n">
         <v>8</v>
@@ -1954,14 +1952,14 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="13" t="n">
+      <c r="A37" s="15" t="n">
         <v>46154</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D37" s="7" t="n">
         <v>38</v>
@@ -1971,14 +1969,14 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="13" t="n">
+      <c r="A38" s="15" t="n">
         <v>46150</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D38" s="7" t="n">
         <v>42</v>
@@ -1988,14 +1986,14 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="13" t="n">
+      <c r="A39" s="15" t="n">
         <v>46065</v>
       </c>
       <c r="B39" s="10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D39" s="7" t="n">
         <v>15</v>
@@ -2005,14 +2003,14 @@
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="13" t="n">
+      <c r="A40" s="15" t="n">
         <v>46048</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D40" s="7" t="n">
         <v>33</v>
@@ -2022,14 +2020,14 @@
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="13" t="n">
+      <c r="A41" s="15" t="n">
         <v>46043</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C41" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D41" s="7" t="n">
         <v>30</v>
@@ -2039,14 +2037,14 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="13" t="n">
+      <c r="A42" s="15" t="n">
         <v>46024</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C42" s="10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D42" s="7" t="n">
         <v>43</v>
@@ -2056,14 +2054,14 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="13" t="n">
+      <c r="A43" s="15" t="n">
         <v>46159</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C43" s="10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D43" s="7" t="n">
         <v>15</v>
@@ -2073,14 +2071,14 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="13" t="n">
+      <c r="A44" s="15" t="n">
         <v>46024</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D44" s="7" t="n">
         <v>30</v>

</xml_diff>